<commit_message>
Update scripts to match new rules and card changes.
</commit_message>
<xml_diff>
--- a/sheet/ItemCardData.xlsx
+++ b/sheet/ItemCardData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27DC2DD6-7EB3-4E70-AF99-6A696CFE7DC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9B4BEFE-331F-467F-9687-8D38494B7FDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t>cardName</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -75,10 +75,6 @@
   </si>
   <si>
     <t>壶</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>tags</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -474,14 +470,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="32.125" customWidth="1"/>
-    <col min="6" max="6" width="62.5" customWidth="1"/>
+    <col min="3" max="3" width="32.125" customWidth="1"/>
+    <col min="5" max="5" width="62.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -489,119 +485,116 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2">
         <v>3</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="2"/>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
       <c r="B3">
         <v>3</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="1:7" ht="42.75" x14ac:dyDescent="0.2">
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="C4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="3"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="2"/>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:6" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="3"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="D6" s="1" t="s">
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="3"/>
-    </row>
-    <row r="7" spans="1:7" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7">
-        <v>3</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="B8">
-        <v>3</v>
-      </c>
-      <c r="D8" s="1" t="s">
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9">
-        <v>3</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>